<commit_message>
Make Leadership Summary recommendations formula-driven and fit it to one printed page
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HWJPGXsj2qYh7Jm78XTTLr
</commit_message>
<xml_diff>
--- a/LastName_FirstName_SS_Modeling_Lab.xlsx
+++ b/LastName_FirstName_SS_Modeling_Lab.xlsx
@@ -6224,6 +6224,9 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{710D3160-0B3E-47E4-AC4A-53506BAB2BA3}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -6443,8 +6446,9 @@
       <c r="F22" s="66"/>
     </row>
     <row r="23" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="70" t="s">
-        <v>144</v>
+      <c r="A23" s="70" t="str">
+        <f>"1. Switch to recycled fabric if you expect to make this hoodie for "&amp;B15&amp;" or more years: it costs "&amp;TEXT('Cost Projection'!G24,"$0.00")&amp;" more now but is cheaper from year "&amp;B15&amp;" and the gap widens."</f>
+        <v>1. Switch to recycled fabric if you expect to make this hoodie for 3 or more years: it costs $1.15 more now but is cheaper from year 3 and the gap widens.</v>
       </c>
       <c r="B23" s="70"/>
       <c r="C23" s="70"/>
@@ -6453,8 +6457,9 @@
       <c r="F23" s="70"/>
     </row>
     <row r="24" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="70" t="s">
-        <v>145</v>
+      <c r="A24" s="70" t="str">
+        <f>"2. Run the campaign, but test a smaller click purchase first to measure the real conversion rate; profit disappears below about "&amp;TEXT('Break-even'!E21,"0.0%")&amp;"."</f>
+        <v>2. Run the campaign, but test a smaller click purchase first to measure the real conversion rate; profit disappears below about 3.4%.</v>
       </c>
       <c r="B24" s="70"/>
       <c r="C24" s="70"/>
@@ -6463,8 +6468,9 @@
       <c r="F24" s="70"/>
     </row>
     <row r="25" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="70" t="s">
-        <v>146</v>
+      <c r="A25" s="70" t="str">
+        <f>"3. Protect the margin: keep the average order near "&amp;TEXT('Break-even'!B13,"$0")&amp;" (break-even is about "&amp;TEXT('Break-even'!E22,"$0.00")&amp;") and watch the cost per click."</f>
+        <v>3. Protect the margin: keep the average order near $60 (break-even is about $55.80) and watch the cost per click.</v>
       </c>
       <c r="B25" s="70"/>
       <c r="C25" s="70"/>
@@ -6493,6 +6499,7 @@
     <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" fitToWidth="1" fitToHeight="1"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>